<commit_message>
swap sidebar: demo links above ticker header
</commit_message>
<xml_diff>
--- a/google search options.xlsx
+++ b/google search options.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebastianflores/Desktop/OpenTF/miteproyects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4024699B-1D33-5B4E-941E-1902A9813DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B416E8D7-4C73-614D-BF08-DADF421E1F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="500" windowWidth="24740" windowHeight="14900" activeTab="1" xr2:uid="{6D825CFA-3F19-CD42-B085-953C484A193E}"/>
+    <workbookView xWindow="60" yWindow="600" windowWidth="24740" windowHeight="14900" activeTab="1" xr2:uid="{6D825CFA-3F19-CD42-B085-953C484A193E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Do not code, lets keep improving this.  Send me your corrections based on limit.  Improve text, context, grammar.</t>
   </si>
@@ -79,6 +79,24 @@
   </si>
   <si>
     <t>This are my choices.  Check limits, do not suggest changes besides limit factor.</t>
+  </si>
+  <si>
+    <t>SITELINK 1: https://quartercharts.com/?page=charts&amp;ticker=NVDA</t>
+  </si>
+  <si>
+    <t>SITELINK 2: https://quartercharts.com/?page=sankey&amp;ticker=NVDA</t>
+  </si>
+  <si>
+    <t>SITELINK 3: https://quartercharts.com/?page=pricing&amp;ticker=NVDA</t>
+  </si>
+  <si>
+    <t>SITELINK 4: https://quartercharts.com/?page=profile&amp;ticker=NVDA</t>
+  </si>
+  <si>
+    <t>send title and description options</t>
+  </si>
+  <si>
+    <t>SITELINK 5: https://quartercharts.com/?page=watchlist&amp;ticker=NVDA</t>
   </si>
 </sst>
 </file>
@@ -525,7 +543,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D8F0A7-387A-B341-B743-B327702DC642}">
-  <dimension ref="B2:B18"/>
+  <dimension ref="B2:B24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.2">
@@ -550,7 +568,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.2">
@@ -565,7 +583,7 @@
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.2">
@@ -580,7 +598,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.2">
@@ -591,6 +609,26 @@
     <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>